<commit_message>
wersja stabilna z zapisem obrazków do katalogu na googdle dri
</commit_message>
<xml_diff>
--- a/prompts/requiem_etapy.xlsx
+++ b/prompts/requiem_etapy.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="etapy" sheetId="1" state="visible" r:id="rId3"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="114">
   <si>
     <t xml:space="preserve">etap</t>
   </si>
@@ -284,6 +284,9 @@
     <t xml:space="preserve">Remonty - wymiana żarówek w gwiazdach</t>
   </si>
   <si>
+    <t xml:space="preserve">drzwi10.png</t>
+  </si>
+  <si>
     <t xml:space="preserve">Remonty - renowacja planet kamiennych</t>
   </si>
   <si>
@@ -303,9 +306,6 @@
   </si>
   <si>
     <t xml:space="preserve">Remonty - instalacja klimatyzacji w Piekle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">drzwi10.png</t>
   </si>
   <si>
     <t xml:space="preserve">Remonty - remont tunelu czasoprzestrzennego</t>
@@ -1481,7 +1481,7 @@
         <v>86</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>69</v>
+        <v>87</v>
       </c>
       <c r="D33" s="7"/>
       <c r="E33" s="7" t="n">
@@ -1496,11 +1496,9 @@
         <v>33</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="C34" s="7" t="s">
-        <v>73</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="C34" s="0"/>
       <c r="D34" s="6"/>
       <c r="E34" s="7" t="n">
         <v>90</v>
@@ -1514,11 +1512,9 @@
         <v>34</v>
       </c>
       <c r="B35" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>75</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="C35" s="6"/>
       <c r="D35" s="7"/>
       <c r="E35" s="7" t="n">
         <v>90</v>
@@ -1532,11 +1528,9 @@
         <v>35</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>79</v>
-      </c>
+        <v>90</v>
+      </c>
+      <c r="C36" s="7"/>
       <c r="D36" s="6"/>
       <c r="E36" s="7" t="n">
         <v>90</v>
@@ -1550,11 +1544,9 @@
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>90</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>81</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="C37" s="0"/>
       <c r="D37" s="7"/>
       <c r="E37" s="7" t="n">
         <v>90</v>
@@ -1568,11 +1560,9 @@
         <v>37</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>83</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="C38" s="0"/>
       <c r="D38" s="6"/>
       <c r="E38" s="7" t="n">
         <v>90</v>
@@ -1586,11 +1576,9 @@
         <v>38</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>85</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="C39" s="0"/>
       <c r="D39" s="7"/>
       <c r="E39" s="7" t="n">
         <v>90</v>
@@ -1604,11 +1592,9 @@
         <v>39</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C40" s="6" t="s">
         <v>94</v>
       </c>
+      <c r="C40" s="0"/>
       <c r="D40" s="6"/>
       <c r="E40" s="7" t="n">
         <v>90</v>

</xml_diff>